<commit_message>
modificaciones de exceles y algoritmo de balanceo
</commit_message>
<xml_diff>
--- a/Tutores/public/templates/NuevoIngreso.xlsx
+++ b/Tutores/public/templates/NuevoIngreso.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shiha\Downloads\▓ Archivos_ProgramaTutoria\PlantillasExcelsCarga\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shiha\Downloads\▓ Archivos_ProgramaTutoria\Excels NUEVA VERSION\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08538BF-6298-4D52-95B1-17E39BD8444D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C32D0CB0-F559-4B36-A90D-B878DEA4689B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D29FC215-4BC9-4888-807F-2E5C8CB05143}"/>
   </bookViews>
@@ -39,19 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>Licenciatura Tutor</t>
-  </si>
-  <si>
-    <t>Nombre del Tutor</t>
-  </si>
-  <si>
-    <t>Apellido Paterno Tutor</t>
-  </si>
-  <si>
-    <t>Apellido Materno Tutor</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Licenciatura Tutorado</t>
   </si>
@@ -78,15 +66,6 @@
   </si>
   <si>
     <t>ICO</t>
-  </si>
-  <si>
-    <t>JUAN</t>
-  </si>
-  <si>
-    <t>SANCHEZ</t>
-  </si>
-  <si>
-    <t>HERRERA</t>
   </si>
   <si>
     <t>Jorge</t>
@@ -134,12 +113,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,10 +452,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5310447A-F454-4C48-B1BE-134486E4DD72}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,13 +463,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -499,52 +477,28 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>4150001</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2">
-        <v>4150001</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>